<commit_message>
Fix MPBF Method II formula to match its label (fixed 25% margin)
Form_V_MPBF row 10 is labelled "MPBF - Method II (0.75*CA - CL)" but its
formula used the variable Assumptions!C55 margin instead of a fixed 0.75,
so the computed MPBF didn't match what the label claimed. Method II is a
banking-standard term (Tandon Committee) with a fixed 25% margin, unlike
Method I's negotiated margin -- so the formula, not the label, was wrong.
Changed C10:G10 (all 5 years) to MAX(0, CA*0.75 - CL).

Verified via zip-level chart/drawing byte comparison that the template
edit didn't disturb any embedded chart/drawing.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/bank_loan/CMA_Dashboard_Premium.xlsx
+++ b/templates/bank_loan/CMA_Dashboard_Premium.xlsx
@@ -4863,23 +4863,23 @@
         </is>
       </c>
       <c r="C10" s="143">
-        <f>MAX(0,Form_IV_CA_CL!C14*(1-Assumptions!$C$55)-Form_IV_CA_CL!C18)</f>
+        <f>MAX(0,Form_IV_CA_CL!C14*0.75-Form_IV_CA_CL!C18)</f>
         <v/>
       </c>
       <c r="D10" s="143">
-        <f>MAX(0,Form_IV_CA_CL!D14*(1-Assumptions!$C$55)-Form_IV_CA_CL!D18)</f>
+        <f>MAX(0,Form_IV_CA_CL!D14*0.75-Form_IV_CA_CL!D18)</f>
         <v/>
       </c>
       <c r="E10" s="143">
-        <f>MAX(0,Form_IV_CA_CL!E14*(1-Assumptions!$C$55)-Form_IV_CA_CL!E18)</f>
+        <f>MAX(0,Form_IV_CA_CL!E14*0.75-Form_IV_CA_CL!E18)</f>
         <v/>
       </c>
       <c r="F10" s="143">
-        <f>MAX(0,Form_IV_CA_CL!F14*(1-Assumptions!$C$55)-Form_IV_CA_CL!F18)</f>
+        <f>MAX(0,Form_IV_CA_CL!F14*0.75-Form_IV_CA_CL!F18)</f>
         <v/>
       </c>
       <c r="G10" s="143">
-        <f>MAX(0,Form_IV_CA_CL!G14*(1-Assumptions!$C$55)-Form_IV_CA_CL!G18)</f>
+        <f>MAX(0,Form_IV_CA_CL!G14*0.75-Form_IV_CA_CL!G18)</f>
         <v/>
       </c>
     </row>
@@ -10872,7 +10872,7 @@
           <t>M12</t>
         </is>
       </c>
-      <c r="O20" t="inlineStr">
+      <c r="O20" s="81" t="inlineStr">
         <is>
           <t>Gestation (months, 0-11)</t>
         </is>
@@ -10946,7 +10946,7 @@
       <c r="L21" s="126" t="n"/>
       <c r="M21" s="126" t="n"/>
       <c r="N21" s="126" t="n"/>
-      <c r="O21" t="n">
+      <c r="O21" s="81" t="n">
         <v>0</v>
       </c>
       <c r="S21" s="81" t="inlineStr">
@@ -11128,12 +11128,12 @@
       </c>
       <c r="D32" s="335" t="n"/>
       <c r="E32" s="336" t="n"/>
-      <c r="F32" t="inlineStr">
+      <c r="F32" s="81" t="inlineStr">
         <is>
           <t>(headcount)</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="G32" s="81" t="inlineStr">
         <is>
           <t>(₹ / employee / month)</t>
         </is>

</xml_diff>

<commit_message>
Add the Cost of Project block to the universal template too
Missed in both the original hotel_cma fix and the subsequent propagation
to the other 9 industry templates: the universal bank_loan_cma workbook
(used by any industry without its own dedicated template -- manufacturing,
agriculture, construction, renewable energy, etc.) never got the block at
all. Caught verifying project 83 (Edible Coffee Cups, a manufacturing
project on the universal template): Assumptions!C81/C86 came back blank
because the cells simply didn't exist there.

Same block, same layout (row 75 is this template's last used row too, no
merges beyond it -- identical to every other template before its own fix),
appended after row 75. Added the matching Pre-operative Expenses schema
field. Verified via a direct fill_template rebuild of project 83's real
stored data (no LLM call): Fixed Assets, Means of Finance and the tie-out
check all compute correctly.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/bank_loan/CMA_Dashboard_Premium.xlsx
+++ b/templates/bank_loan/CMA_Dashboard_Premium.xlsx
@@ -3563,7 +3563,7 @@
           <t>DSCR</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="81" t="inlineStr">
         <is>
           <t>Debt-service coverage year by year</t>
         </is>
@@ -3611,9 +3611,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="B12:C12"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B12:C12"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B13" location="Assumptions!A1" display="Assumptions"/>
@@ -9526,7 +9526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AF75"/>
+  <dimension ref="A1:AF87"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.71484375" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="81" min="1" max="1"/>
@@ -11724,6 +11724,142 @@
         <is>
           <t>months</t>
         </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>K.  COST OF PROJECT  (bottom-up build-up; ties to Means of Finance below)</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Fixed assets (land + building + plant &amp; machinery + furniture)</t>
+        </is>
+      </c>
+      <c r="C78">
+        <f>C42+C43+C45+C47</f>
+        <v/>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>₹</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Pre-operative &amp; preliminary expenses</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>0</v>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>₹</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Margin money for working capital  (borrower's stipulated NWC, Year 1)</t>
+        </is>
+      </c>
+      <c r="C80">
+        <f>'WC &amp; CC-OD Limit'!C10</f>
+        <v/>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>₹</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>TOTAL PROJECT COST</t>
+        </is>
+      </c>
+      <c r="C81">
+        <f>C78+C79+C80</f>
+        <v/>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>₹</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>MEANS OF FINANCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Term loan</t>
+        </is>
+      </c>
+      <c r="C84">
+        <f>C8</f>
+        <v/>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>₹</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Promoter's contribution</t>
+        </is>
+      </c>
+      <c r="C85">
+        <f>C9</f>
+        <v/>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>₹</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>TOTAL MEANS OF FINANCE</t>
+        </is>
+      </c>
+      <c r="C86">
+        <f>C84+C85</f>
+        <v/>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>₹</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Check  (Total Project Cost − Total Means of Finance = 0)</t>
+        </is>
+      </c>
+      <c r="C87">
+        <f>C81-C86</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>